<commit_message>
Saída: edição 2026-09 refeita com o código de outubro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
(cherry picked from commit 75856d66fc012ed78e3c20b82020a3d276fbd76a)
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/_Historico/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/_Historico/2026-09/conferencia_2026-09.xlsx
@@ -5279,7 +5279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -5599,20 +5599,42 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>prevtopcredit</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tivio Prev Top Credit Itaú</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>comentário do gestor</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>não preenchido no arquivo de comentários</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>atuarial</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Tivio Atuarial</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>rentabilidade</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>sem cotas na dados_mensais</t>
         </is>
@@ -5712,12 +5734,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K133"/>
+  <dimension ref="A1:K139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -10708,17 +10730,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevtopcredit</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Top Credit Itaú</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREVIDENCIA TOP CREDIT ITAÚ I FIF CIC RF CP RL - Expandida</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -10735,35 +10757,35 @@
         <v>46265</v>
       </c>
       <c r="G116" t="n">
-        <v>-0.001462081025388806</v>
+        <v>0.01013823405235592</v>
       </c>
       <c r="H116" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I116" t="n">
-        <v>-0.01228767290543542</v>
+        <v>-0.0006873578276906933</v>
       </c>
       <c r="J116" t="n">
-        <v>-0.1350578371685771</v>
+        <v>0.9365062127496595</v>
       </c>
       <c r="K116" t="n">
-        <v>-0.1365046674965383</v>
+        <v>-0.00812950854763983</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevtopcredit</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Top Credit Itaú</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREVIDENCIA TOP CREDIT ITAÚ I FIF CIC RF CP RL - Expandida</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -10780,35 +10802,35 @@
         <v>46022</v>
       </c>
       <c r="G117" t="n">
-        <v>0.08638432471204283</v>
+        <v>0.09863687152086498</v>
       </c>
       <c r="H117" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I117" t="n">
-        <v>-0.01872845997810102</v>
+        <v>-0.006475913169278869</v>
       </c>
       <c r="J117" t="n">
-        <v>0.8218250992654261</v>
+        <v>0.9383908133690031</v>
       </c>
       <c r="K117" t="n">
-        <v>-0.0227702919562276</v>
+        <v>-0.007888787424651156</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevtopcredit</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Top Credit Itaú</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREVIDENCIA TOP CREDIT ITAÚ I FIF CIC RF CP RL - Expandida</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -10822,28 +10844,38 @@
         </is>
       </c>
       <c r="F118" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
+        <v>45930</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0.1352362052012954</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0.1447903912030524</v>
+      </c>
+      <c r="I118" t="n">
+        <v>-0.009554186001756948</v>
+      </c>
+      <c r="J118" t="n">
+        <v>0.9340136736811612</v>
+      </c>
+      <c r="K118" t="n">
+        <v>-0.008378905558415473</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevtopcredit</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Top Credit Itaú</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREVIDENCIA TOP CREDIT ITAÚ I FIF CIC RF CP RL - Expandida</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -10857,28 +10889,38 @@
         </is>
       </c>
       <c r="F119" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
+        <v>45561</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0.2737092175629274</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0.2980670513506256</v>
+      </c>
+      <c r="I119" t="n">
+        <v>-0.02435783378769818</v>
+      </c>
+      <c r="J119" t="n">
+        <v>0.9182806899409848</v>
+      </c>
+      <c r="K119" t="n">
+        <v>-0.009445432486984373</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevtopcredit</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Top Credit Itaú</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREVIDENCIA TOP CREDIT ITAÚ I FIF CIC RF CP RL - Expandida</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -10892,28 +10934,38 @@
         </is>
       </c>
       <c r="F120" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
+        <v>45195</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0.4359288220235673</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0.4424561999402108</v>
+      </c>
+      <c r="I120" t="n">
+        <v>-0.006527377916643484</v>
+      </c>
+      <c r="J120" t="n">
+        <v>0.9852474032061805</v>
+      </c>
+      <c r="K120" t="n">
+        <v>-0.001512674621442001</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevtopcredit</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Top Credit Itaú</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREVIDENCIA TOP CREDIT ITAÚ I FIF CIC RF CP RL - Expandida</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -10927,43 +10979,43 @@
         </is>
       </c>
       <c r="F121" s="1" t="n">
-        <v>45950</v>
+        <v>44861</v>
       </c>
       <c r="G121" t="n">
-        <v>0.1194341999999999</v>
+        <v>0.5731109999999999</v>
       </c>
       <c r="H121" t="n">
-        <v>0.1359909271883835</v>
+        <v>0.6191840248450784</v>
       </c>
       <c r="I121" t="n">
-        <v>-0.01655672718838352</v>
+        <v>-0.04607302484507847</v>
       </c>
       <c r="J121" t="n">
-        <v>0.8782512368237032</v>
+        <v>0.9255907403996638</v>
       </c>
       <c r="K121" t="n">
-        <v>-0.0154899691480026</v>
+        <v>-0.00736554626356889</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -10975,40 +11027,40 @@
         <v>46265</v>
       </c>
       <c r="G122" t="n">
-        <v>0.01003070736812051</v>
+        <v>-0.001462081025388806</v>
       </c>
       <c r="H122" t="n">
-        <v>0.0200519906458918</v>
+        <v>0.01082559188004661</v>
       </c>
       <c r="I122" t="n">
-        <v>-0.0100212832777713</v>
+        <v>-0.01228767290543542</v>
       </c>
       <c r="J122" t="n">
-        <v>0.5002349913910203</v>
+        <v>-0.1350578371685771</v>
       </c>
       <c r="K122" t="n">
-        <v>-0.1117254109753738</v>
+        <v>-0.1365046674965383</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -11020,40 +11072,40 @@
         <v>46022</v>
       </c>
       <c r="G123" t="n">
-        <v>0.07172731728642034</v>
+        <v>0.08638432471204283</v>
       </c>
       <c r="H123" t="n">
-        <v>0.1136619152554992</v>
+        <v>0.1051127846901438</v>
       </c>
       <c r="I123" t="n">
-        <v>-0.04193459796907884</v>
+        <v>-0.01872845997810102</v>
       </c>
       <c r="J123" t="n">
-        <v>0.6310584959367033</v>
+        <v>0.8218250992654261</v>
       </c>
       <c r="K123" t="n">
-        <v>-0.05040838364525002</v>
+        <v>-0.0227702919562276</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -11062,43 +11114,33 @@
         </is>
       </c>
       <c r="F124" s="1" t="n">
-        <v>45930</v>
-      </c>
-      <c r="G124" t="n">
-        <v>0.09357535556093843</v>
-      </c>
-      <c r="H124" t="n">
-        <v>0.1479693332684646</v>
-      </c>
-      <c r="I124" t="n">
-        <v>-0.05439397770752619</v>
-      </c>
-      <c r="J124" t="n">
-        <v>0.6323969534360354</v>
-      </c>
-      <c r="K124" t="n">
-        <v>-0.0475669929009177</v>
-      </c>
+        <v>45950</v>
+      </c>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -11107,7 +11149,7 @@
         </is>
       </c>
       <c r="F125" s="1" t="n">
-        <v>45586</v>
+        <v>45950</v>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
@@ -11118,22 +11160,22 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -11142,7 +11184,7 @@
         </is>
       </c>
       <c r="F126" s="1" t="n">
-        <v>45586</v>
+        <v>45950</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr"/>
@@ -11153,22 +11195,22 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -11177,43 +11219,43 @@
         </is>
       </c>
       <c r="F127" s="1" t="n">
-        <v>45586</v>
+        <v>45950</v>
       </c>
       <c r="G127" t="n">
-        <v>0.2135222000000001</v>
+        <v>0.1194341999999999</v>
       </c>
       <c r="H127" t="n">
-        <v>0.2465452463189715</v>
+        <v>0.1359909271883835</v>
       </c>
       <c r="I127" t="n">
-        <v>-0.03302304631897135</v>
+        <v>-0.01655672718838352</v>
       </c>
       <c r="J127" t="n">
-        <v>0.8660568523951693</v>
+        <v>0.8782512368237032</v>
       </c>
       <c r="K127" t="n">
-        <v>-0.01382518449086667</v>
+        <v>-0.0154899691480026</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -11225,40 +11267,40 @@
         <v>46265</v>
       </c>
       <c r="G128" t="n">
-        <v>0.01025992096101835</v>
+        <v>0.01003070736812051</v>
       </c>
       <c r="H128" t="n">
-        <v>0.01082559188004661</v>
+        <v>0.0200519906458918</v>
       </c>
       <c r="I128" t="n">
-        <v>-0.0005656709190282605</v>
+        <v>-0.0100212832777713</v>
       </c>
       <c r="J128" t="n">
-        <v>0.9477468830068416</v>
+        <v>0.5002349913910203</v>
       </c>
       <c r="K128" t="n">
-        <v>-0.006694722873975767</v>
+        <v>-0.1117254109753738</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -11270,40 +11312,40 @@
         <v>46022</v>
       </c>
       <c r="G129" t="n">
-        <v>0.1002856499041807</v>
+        <v>0.07172731728642034</v>
       </c>
       <c r="H129" t="n">
-        <v>0.1051127846901438</v>
+        <v>0.1136619152554992</v>
       </c>
       <c r="I129" t="n">
-        <v>-0.004827134785963194</v>
+        <v>-0.04193459796907884</v>
       </c>
       <c r="J129" t="n">
-        <v>0.9540766158922263</v>
+        <v>0.6310584959367033</v>
       </c>
       <c r="K129" t="n">
-        <v>-0.00588181858317427</v>
+        <v>-0.05040838364525002</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -11315,40 +11357,40 @@
         <v>45930</v>
       </c>
       <c r="G130" t="n">
-        <v>0.1394310574216069</v>
+        <v>0.09357535556093843</v>
       </c>
       <c r="H130" t="n">
-        <v>0.1447903912030524</v>
+        <v>0.1479693332684646</v>
       </c>
       <c r="I130" t="n">
-        <v>-0.005359333781445486</v>
+        <v>-0.05439397770752619</v>
       </c>
       <c r="J130" t="n">
-        <v>0.9629855701271667</v>
+        <v>0.6323969534360354</v>
       </c>
       <c r="K130" t="n">
-        <v>-0.004700105358509954</v>
+        <v>-0.0475669929009177</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -11357,43 +11399,33 @@
         </is>
       </c>
       <c r="F131" s="1" t="n">
-        <v>45561</v>
-      </c>
-      <c r="G131" t="n">
-        <v>0.288834593654415</v>
-      </c>
-      <c r="H131" t="n">
-        <v>0.2980670513506256</v>
-      </c>
-      <c r="I131" t="n">
-        <v>-0.009232457696210616</v>
-      </c>
-      <c r="J131" t="n">
-        <v>0.9690255677225116</v>
-      </c>
-      <c r="K131" t="n">
-        <v>-0.00356964896216394</v>
-      </c>
+        <v>45586</v>
+      </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -11402,66 +11434,326 @@
         </is>
       </c>
       <c r="F132" s="1" t="n">
-        <v>45195</v>
-      </c>
-      <c r="G132" t="n">
-        <v>0.4630786945344103</v>
-      </c>
-      <c r="H132" t="n">
-        <v>0.4424561999402108</v>
-      </c>
-      <c r="I132" t="n">
-        <v>0.02062249459419951</v>
-      </c>
-      <c r="J132" t="n">
-        <v>1.046609121076812</v>
-      </c>
-      <c r="K132" t="n">
-        <v>0.004749361817451225</v>
-      </c>
+        <v>45586</v>
+      </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>IMA-B 5</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>inicio</t>
+        </is>
+      </c>
+      <c r="F133" s="1" t="n">
+        <v>45586</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0.2135222000000001</v>
+      </c>
+      <c r="H133" t="n">
+        <v>0.2465452463189715</v>
+      </c>
+      <c r="I133" t="n">
+        <v>-0.03302304631897135</v>
+      </c>
+      <c r="J133" t="n">
+        <v>0.8660568523951693</v>
+      </c>
+      <c r="K133" t="n">
+        <v>-0.01382518449086667</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
           <t>legacy</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
+      <c r="B134" t="inlineStr">
         <is>
           <t>Tivio Legacy Prev</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
+      <c r="C134" t="inlineStr">
         <is>
           <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
         </is>
       </c>
-      <c r="D133" t="inlineStr">
+      <c r="D134" t="inlineStr">
         <is>
           <t>CDI</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr">
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="F134" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="G134" t="n">
+        <v>0.01025992096101835</v>
+      </c>
+      <c r="H134" t="n">
+        <v>0.01082559188004661</v>
+      </c>
+      <c r="I134" t="n">
+        <v>-0.0005656709190282605</v>
+      </c>
+      <c r="J134" t="n">
+        <v>0.9477468830068416</v>
+      </c>
+      <c r="K134" t="n">
+        <v>-0.006694722873975767</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="F135" s="1" t="n">
+        <v>46022</v>
+      </c>
+      <c r="G135" t="n">
+        <v>0.1002856499041807</v>
+      </c>
+      <c r="H135" t="n">
+        <v>0.1051127846901438</v>
+      </c>
+      <c r="I135" t="n">
+        <v>-0.004827134785963194</v>
+      </c>
+      <c r="J135" t="n">
+        <v>0.9540766158922263</v>
+      </c>
+      <c r="K135" t="n">
+        <v>-0.00588181858317427</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>12m</t>
+        </is>
+      </c>
+      <c r="F136" s="1" t="n">
+        <v>45930</v>
+      </c>
+      <c r="G136" t="n">
+        <v>0.1394310574216069</v>
+      </c>
+      <c r="H136" t="n">
+        <v>0.1447903912030524</v>
+      </c>
+      <c r="I136" t="n">
+        <v>-0.005359333781445486</v>
+      </c>
+      <c r="J136" t="n">
+        <v>0.9629855701271667</v>
+      </c>
+      <c r="K136" t="n">
+        <v>-0.004700105358509954</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>24m</t>
+        </is>
+      </c>
+      <c r="F137" s="1" t="n">
+        <v>45561</v>
+      </c>
+      <c r="G137" t="n">
+        <v>0.288834593654415</v>
+      </c>
+      <c r="H137" t="n">
+        <v>0.2980670513506256</v>
+      </c>
+      <c r="I137" t="n">
+        <v>-0.009232457696210616</v>
+      </c>
+      <c r="J137" t="n">
+        <v>0.9690255677225116</v>
+      </c>
+      <c r="K137" t="n">
+        <v>-0.00356964896216394</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>36m</t>
+        </is>
+      </c>
+      <c r="F138" s="1" t="n">
+        <v>45195</v>
+      </c>
+      <c r="G138" t="n">
+        <v>0.4630786945344103</v>
+      </c>
+      <c r="H138" t="n">
+        <v>0.4424561999402108</v>
+      </c>
+      <c r="I138" t="n">
+        <v>0.02062249459419951</v>
+      </c>
+      <c r="J138" t="n">
+        <v>1.046609121076812</v>
+      </c>
+      <c r="K138" t="n">
+        <v>0.004749361817451225</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
         <is>
           <t>inicio</t>
         </is>
       </c>
-      <c r="F133" s="1" t="n">
+      <c r="F139" s="1" t="n">
         <v>39674</v>
       </c>
-      <c r="G133" t="n">
+      <c r="G139" t="n">
         <v>4.4092549</v>
       </c>
-      <c r="H133" t="n">
+      <c r="H139" t="n">
         <v>4.604775473331634</v>
       </c>
-      <c r="I133" t="n">
+      <c r="I139" t="n">
         <v>-0.1955205733316348</v>
       </c>
-      <c r="J133" t="n">
+      <c r="J139" t="n">
         <v>0.957539607639073</v>
       </c>
-      <c r="K133" t="n">
+      <c r="K139" t="n">
         <v>-0.001963351321792373</v>
       </c>
     </row>
@@ -11476,7 +11768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12122,22 +12414,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevtopcredit</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Top Credit Itaú</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>62.791.756/0001-53</t>
+          <t>42.535.150/0001-40</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,75% a.a.</t>
+          <t>0,80% a.a.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -12154,22 +12446,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>54.853.793/0001-10</t>
+          <t>62.791.756/0001-53</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,475% a.a.</t>
+          <t>0,75% a.a.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -12186,30 +12478,62 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>54.853.793/0001-10</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0,475% a.a.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Não há</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>legacy</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Tivio Legacy Prev</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>09.083.848/0001-04</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>0,50% a.a.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Não há</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>não</t>
         </is>
@@ -12226,7 +12550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -12276,12 +12600,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>conexaoalt180</t>
+          <t>indicadores</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>sem carteira na Base Carteira — alocação, carrego e duration mantidos</t>
+          <t>JSON do Informativo ausente. Atualize data/tivio_summary.json (procurado em C:\Users\renan\OneDrive\Documentos\_all\CHAVES\Projetos\Tivio Capital\AutomaTivio\data\tivio_summary.json). AUM por vertical ficou como no modelo.</t>
         </is>
       </c>
     </row>
@@ -12293,53 +12617,53 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>conexaoalt180</t>
+          <t>indicadores</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>taxa global não encontrada na taxas_global.xlsx</t>
+          <t>anos_historia forçado em configs/big_numbers.yml: a fonte oficial diz +25, o material usa +27. Tire a linha de `forcar:` quando a fonte for corrigida.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>relatorio/bvp</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bvp</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
+          <t>sem carteira na Base Carteira — alocação, carrego e duration mantidos</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>relatorio/atuarial</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>atuarial</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>relatório não gerado: sem dados nesta edição</t>
+          <t>taxa global não encontrada na taxas_global.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>relatorio/credito_privado</t>
+          <t>relatorio/bvp</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -12356,41 +12680,41 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>landing/hgd30</t>
+          <t>relatorio/atuarial</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>atuarial</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
+          <t>relatório não gerado: sem dados nesta edição</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>landing/hyd60</t>
+          <t>relatorio/credito_privado</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>bvp</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>email/previdencia</t>
+          <t>landing/hgd30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -12407,7 +12731,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>email/previdencia</t>
+          <t>landing/hyd60</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -12424,51 +12748,51 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>email/previdencia</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>email/previdencia</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
         </is>
       </c>
     </row>
@@ -12520,6 +12844,57 @@
       <c r="C17" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>decks</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>taxas_prev</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ALTLIGHT: FIE I: Custódia = 1720.46 (fora do padrão de percentual)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>decks</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>prevlowvol</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>deck: sem comentário em entrada/comentarios.md, saiu lorem ipsum</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>decks</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>prevtopcredit</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>deck: sem comentário em entrada/comentarios.md, saiu lorem ipsum</t>
         </is>
       </c>
     </row>
@@ -12534,7 +12909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -13201,7 +13576,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4829406</v>
+        <v>4829399</v>
       </c>
     </row>
     <row r="45">
@@ -13261,7 +13636,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16816512</v>
+        <v>16816508</v>
       </c>
     </row>
     <row r="49">
@@ -13276,7 +13651,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3009396</v>
+        <v>3009388</v>
       </c>
     </row>
     <row r="50">
@@ -13306,7 +13681,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2616247</v>
+        <v>2616224</v>
       </c>
     </row>
     <row r="52">
@@ -13321,7 +13696,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>15041376</v>
+        <v>15041374</v>
       </c>
     </row>
     <row r="53">
@@ -13336,7 +13711,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2467250</v>
+        <v>2467257</v>
       </c>
     </row>
     <row r="54">
@@ -13351,7 +13726,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>25551964</v>
+        <v>25551962</v>
       </c>
     </row>
     <row r="55">
@@ -13366,7 +13741,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2649979</v>
+        <v>2649967</v>
       </c>
     </row>
     <row r="56">
@@ -13381,7 +13756,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>23546226</v>
+        <v>23546223</v>
       </c>
     </row>
     <row r="57">
@@ -13396,7 +13771,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2643349</v>
+        <v>2643339</v>
       </c>
     </row>
     <row r="58">
@@ -13411,7 +13786,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>26316560</v>
+        <v>26316559</v>
       </c>
     </row>
     <row r="59">
@@ -13426,7 +13801,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>4115895</v>
+        <v>4115810</v>
       </c>
     </row>
     <row r="60">
@@ -13441,7 +13816,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>26316812</v>
+        <v>26316813</v>
       </c>
     </row>
     <row r="61">
@@ -13456,7 +13831,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4116719</v>
+        <v>4116613</v>
       </c>
     </row>
     <row r="62">
@@ -13471,7 +13846,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>26457371</v>
+        <v>26457367</v>
       </c>
     </row>
     <row r="63">
@@ -13486,7 +13861,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3802493</v>
+        <v>3802398</v>
       </c>
     </row>
     <row r="64">
@@ -13501,7 +13876,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>26317596</v>
+        <v>26317594</v>
       </c>
     </row>
     <row r="65">
@@ -13516,7 +13891,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3976310</v>
+        <v>3976292</v>
       </c>
     </row>
     <row r="66">
@@ -13531,7 +13906,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>87883503</v>
+        <v>87883490</v>
       </c>
     </row>
     <row r="67">
@@ -13546,21 +13921,261 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>5089352</v>
+        <v>5093112</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>Deck - Tivio Institucional - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>15446309</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Institucional - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>1197486</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Institucional 15 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>19922364</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Institucional 15 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>1158525</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Institucional 30 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>16178935</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Institucional 30 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>1232221</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Infra Plus CDI - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>17338368</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Infra Plus CDI - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>1435747</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Deck - Tivio HGD30 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>33215313</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Deck - Tivio HGD30 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>755608</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Deck - Tivio HYD60 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>25866085</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Deck - Tivio HYD60 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>1091356</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Prev Low Vol - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>4501586</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Prev Low Vol - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>315710</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Prev Top Credit - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>4215058</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Deck - Tivio Prev Top Credit - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>238900</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>index.html</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>html</t>
         </is>
       </c>
-      <c r="C68" t="n">
+      <c r="C84" t="n">
         <v>394</v>
       </c>
     </row>

</xml_diff>